<commit_message>
feat: add blocks 38-48 (without 42 43) 34 31 30 8 63 5 38 3 21 22 11 7 65 4
</commit_message>
<xml_diff>
--- a/src/data/ruse-blocks.xlsx
+++ b/src/data/ruse-blocks.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2718" uniqueCount="1675">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2719" uniqueCount="1676">
   <si>
     <t>Дружба 1</t>
   </si>
@@ -5039,13 +5039,16 @@
   </si>
   <si>
     <t>ул. Бели Брези 103</t>
+  </si>
+  <si>
+    <t>БЛОК 15 ГО НЯМА В ДАННИТЕ</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -5053,8 +5056,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5064,6 +5073,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -5080,9 +5095,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5414,7 +5430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C986"/>
+  <dimension ref="A1:D986"/>
   <sheetFormatPr defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="15.5" customWidth="1"/>
@@ -8062,7 +8078,7 @@
         <v>1486</v>
       </c>
     </row>
-    <row r="241" spans="1:3">
+    <row r="241" spans="1:4">
       <c r="A241" t="s">
         <v>8</v>
       </c>
@@ -8073,7 +8089,7 @@
         <v>1490</v>
       </c>
     </row>
-    <row r="242" spans="1:3">
+    <row r="242" spans="1:4">
       <c r="A242" t="s">
         <v>8</v>
       </c>
@@ -8084,7 +8100,7 @@
         <v>1493</v>
       </c>
     </row>
-    <row r="243" spans="1:3">
+    <row r="243" spans="1:4">
       <c r="A243" t="s">
         <v>8</v>
       </c>
@@ -8095,7 +8111,7 @@
         <v>1497</v>
       </c>
     </row>
-    <row r="244" spans="1:3">
+    <row r="244" spans="1:4">
       <c r="A244" t="s">
         <v>8</v>
       </c>
@@ -8106,18 +8122,21 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="245" spans="1:3">
+    <row r="245" spans="1:4">
       <c r="A245" t="s">
         <v>8</v>
       </c>
-      <c r="B245">
+      <c r="B245" s="2">
         <v>15</v>
       </c>
       <c r="C245" t="s">
         <v>1503</v>
       </c>
-    </row>
-    <row r="246" spans="1:3">
+      <c r="D245" t="s">
+        <v>1675</v>
+      </c>
+    </row>
+    <row r="246" spans="1:4">
       <c r="A246" t="s">
         <v>8</v>
       </c>
@@ -8128,7 +8147,7 @@
         <v>1506</v>
       </c>
     </row>
-    <row r="247" spans="1:3">
+    <row r="247" spans="1:4">
       <c r="A247" t="s">
         <v>8</v>
       </c>
@@ -8139,7 +8158,7 @@
         <v>1508</v>
       </c>
     </row>
-    <row r="248" spans="1:3">
+    <row r="248" spans="1:4">
       <c r="A248" t="s">
         <v>8</v>
       </c>
@@ -8150,7 +8169,7 @@
         <v>1510</v>
       </c>
     </row>
-    <row r="249" spans="1:3">
+    <row r="249" spans="1:4">
       <c r="A249" t="s">
         <v>8</v>
       </c>
@@ -8161,7 +8180,7 @@
         <v>1512</v>
       </c>
     </row>
-    <row r="250" spans="1:3">
+    <row r="250" spans="1:4">
       <c r="A250" t="s">
         <v>8</v>
       </c>
@@ -8172,7 +8191,7 @@
         <v>1514</v>
       </c>
     </row>
-    <row r="251" spans="1:3">
+    <row r="251" spans="1:4">
       <c r="A251" t="s">
         <v>8</v>
       </c>
@@ -8183,7 +8202,7 @@
         <v>1517</v>
       </c>
     </row>
-    <row r="252" spans="1:3">
+    <row r="252" spans="1:4">
       <c r="A252" t="s">
         <v>8</v>
       </c>
@@ -8194,7 +8213,7 @@
         <v>1520</v>
       </c>
     </row>
-    <row r="253" spans="1:3">
+    <row r="253" spans="1:4">
       <c r="A253" t="s">
         <v>8</v>
       </c>
@@ -8205,7 +8224,7 @@
         <v>1522</v>
       </c>
     </row>
-    <row r="254" spans="1:3">
+    <row r="254" spans="1:4">
       <c r="A254" t="s">
         <v>8</v>
       </c>
@@ -8216,7 +8235,7 @@
         <v>1524</v>
       </c>
     </row>
-    <row r="255" spans="1:3">
+    <row r="255" spans="1:4">
       <c r="A255" t="s">
         <v>8</v>
       </c>
@@ -8227,7 +8246,7 @@
         <v>1526</v>
       </c>
     </row>
-    <row r="256" spans="1:3">
+    <row r="256" spans="1:4">
       <c r="A256" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
feat: add zdravec numbers without 52-28
</commit_message>
<xml_diff>
--- a/src/data/ruse-blocks.xlsx
+++ b/src/data/ruse-blocks.xlsx
@@ -7994,7 +7994,7 @@
       <c r="A233" t="s">
         <v>8</v>
       </c>
-      <c r="B233">
+      <c r="B233" s="1">
         <v>3</v>
       </c>
       <c r="C233" t="s">
@@ -8005,7 +8005,7 @@
       <c r="A234" t="s">
         <v>8</v>
       </c>
-      <c r="B234">
+      <c r="B234" s="1">
         <v>4</v>
       </c>
       <c r="C234" t="s">
@@ -8016,7 +8016,7 @@
       <c r="A235" t="s">
         <v>8</v>
       </c>
-      <c r="B235">
+      <c r="B235" s="1">
         <v>5</v>
       </c>
       <c r="C235" t="s">
@@ -8038,7 +8038,7 @@
       <c r="A237" t="s">
         <v>8</v>
       </c>
-      <c r="B237">
+      <c r="B237" s="1">
         <v>7</v>
       </c>
       <c r="C237" t="s">
@@ -8049,7 +8049,7 @@
       <c r="A238" t="s">
         <v>8</v>
       </c>
-      <c r="B238">
+      <c r="B238" s="1">
         <v>8</v>
       </c>
       <c r="C238" t="s">
@@ -8082,7 +8082,7 @@
       <c r="A241" t="s">
         <v>8</v>
       </c>
-      <c r="B241">
+      <c r="B241" s="1">
         <v>11</v>
       </c>
       <c r="C241" t="s">
@@ -8195,7 +8195,7 @@
       <c r="A251" t="s">
         <v>8</v>
       </c>
-      <c r="B251">
+      <c r="B251" s="1">
         <v>21</v>
       </c>
       <c r="C251" t="s">
@@ -8206,7 +8206,7 @@
       <c r="A252" t="s">
         <v>8</v>
       </c>
-      <c r="B252">
+      <c r="B252" s="1">
         <v>22</v>
       </c>
       <c r="C252" t="s">
@@ -8283,7 +8283,7 @@
       <c r="A259" t="s">
         <v>8</v>
       </c>
-      <c r="B259">
+      <c r="B259" s="1">
         <v>30</v>
       </c>
       <c r="C259" t="s">
@@ -8294,7 +8294,7 @@
       <c r="A260" t="s">
         <v>8</v>
       </c>
-      <c r="B260">
+      <c r="B260" s="1">
         <v>31</v>
       </c>
       <c r="C260" t="s">
@@ -8305,7 +8305,7 @@
       <c r="A261" t="s">
         <v>8</v>
       </c>
-      <c r="B261">
+      <c r="B261" s="1">
         <v>34</v>
       </c>
       <c r="C261" t="s">
@@ -8327,7 +8327,7 @@
       <c r="A263" t="s">
         <v>8</v>
       </c>
-      <c r="B263">
+      <c r="B263" s="1">
         <v>36</v>
       </c>
       <c r="C263" t="s">
@@ -8338,7 +8338,7 @@
       <c r="A264" t="s">
         <v>8</v>
       </c>
-      <c r="B264">
+      <c r="B264" s="1">
         <v>38</v>
       </c>
       <c r="C264" t="s">
@@ -8349,7 +8349,7 @@
       <c r="A265" t="s">
         <v>8</v>
       </c>
-      <c r="B265">
+      <c r="B265" s="1">
         <v>39</v>
       </c>
       <c r="C265" t="s">
@@ -8360,7 +8360,7 @@
       <c r="A266" t="s">
         <v>8</v>
       </c>
-      <c r="B266">
+      <c r="B266" s="1">
         <v>40</v>
       </c>
       <c r="C266" t="s">
@@ -8371,7 +8371,7 @@
       <c r="A267" t="s">
         <v>8</v>
       </c>
-      <c r="B267">
+      <c r="B267" s="1">
         <v>41</v>
       </c>
       <c r="C267" t="s">
@@ -8404,7 +8404,7 @@
       <c r="A270" t="s">
         <v>8</v>
       </c>
-      <c r="B270">
+      <c r="B270" s="1">
         <v>44</v>
       </c>
       <c r="C270" t="s">
@@ -8415,7 +8415,7 @@
       <c r="A271" t="s">
         <v>8</v>
       </c>
-      <c r="B271">
+      <c r="B271" s="1">
         <v>45</v>
       </c>
       <c r="C271" t="s">
@@ -8426,7 +8426,7 @@
       <c r="A272" t="s">
         <v>8</v>
       </c>
-      <c r="B272">
+      <c r="B272" s="1">
         <v>46</v>
       </c>
       <c r="C272" t="s">
@@ -8437,7 +8437,7 @@
       <c r="A273" t="s">
         <v>8</v>
       </c>
-      <c r="B273">
+      <c r="B273" s="1">
         <v>47</v>
       </c>
       <c r="C273" t="s">
@@ -8448,7 +8448,7 @@
       <c r="A274" t="s">
         <v>8</v>
       </c>
-      <c r="B274">
+      <c r="B274" s="1">
         <v>48</v>
       </c>
       <c r="C274" t="s">
@@ -8558,7 +8558,7 @@
       <c r="A284" t="s">
         <v>8</v>
       </c>
-      <c r="B284">
+      <c r="B284" s="1">
         <v>63</v>
       </c>
       <c r="C284" t="s">
@@ -8569,7 +8569,7 @@
       <c r="A285" t="s">
         <v>8</v>
       </c>
-      <c r="B285">
+      <c r="B285" s="1">
         <v>65</v>
       </c>
       <c r="C285" t="s">
@@ -8822,7 +8822,7 @@
       <c r="A308" t="s">
         <v>8</v>
       </c>
-      <c r="B308">
+      <c r="B308" s="1">
         <v>131</v>
       </c>
       <c r="C308" t="s">

</xml_diff>

<commit_message>
feat: sync up spreadsheet
</commit_message>
<xml_diff>
--- a/src/data/ruse-blocks.xlsx
+++ b/src/data/ruse-blocks.xlsx
@@ -9103,7 +9103,7 @@
       <c r="A331" t="s">
         <v>117</v>
       </c>
-      <c r="B331" t="s">
+      <c r="B331" s="1" t="s">
         <v>118</v>
       </c>
       <c r="C331" t="s">
@@ -9114,7 +9114,7 @@
       <c r="A332" t="s">
         <v>117</v>
       </c>
-      <c r="B332" t="s">
+      <c r="B332" s="1" t="s">
         <v>394</v>
       </c>
       <c r="C332" t="s">
@@ -9125,7 +9125,7 @@
       <c r="A333" t="s">
         <v>117</v>
       </c>
-      <c r="B333" t="s">
+      <c r="B333" s="1" t="s">
         <v>816</v>
       </c>
       <c r="C333" t="s">
@@ -9136,7 +9136,7 @@
       <c r="A334" t="s">
         <v>117</v>
       </c>
-      <c r="B334" t="s">
+      <c r="B334" s="1" t="s">
         <v>888</v>
       </c>
       <c r="C334" t="s">
@@ -9147,7 +9147,7 @@
       <c r="A335" t="s">
         <v>117</v>
       </c>
-      <c r="B335" t="s">
+      <c r="B335" s="1" t="s">
         <v>990</v>
       </c>
       <c r="C335" t="s">
@@ -9158,7 +9158,7 @@
       <c r="A336" t="s">
         <v>117</v>
       </c>
-      <c r="B336" t="s">
+      <c r="B336" s="1" t="s">
         <v>1018</v>
       </c>
       <c r="C336" t="s">
@@ -9169,7 +9169,7 @@
       <c r="A337" t="s">
         <v>117</v>
       </c>
-      <c r="B337" t="s">
+      <c r="B337" s="1" t="s">
         <v>1102</v>
       </c>
       <c r="C337" t="s">
@@ -9180,7 +9180,7 @@
       <c r="A338" t="s">
         <v>117</v>
       </c>
-      <c r="B338" t="s">
+      <c r="B338" s="1" t="s">
         <v>1106</v>
       </c>
       <c r="C338" t="s">
@@ -9191,7 +9191,7 @@
       <c r="A339" t="s">
         <v>117</v>
       </c>
-      <c r="B339" t="s">
+      <c r="B339" s="1" t="s">
         <v>1126</v>
       </c>
       <c r="C339" t="s">
@@ -9202,7 +9202,7 @@
       <c r="A340" t="s">
         <v>117</v>
       </c>
-      <c r="B340" t="s">
+      <c r="B340" s="1" t="s">
         <v>1130</v>
       </c>
       <c r="C340" t="s">
@@ -9213,7 +9213,7 @@
       <c r="A341" t="s">
         <v>117</v>
       </c>
-      <c r="B341" t="s">
+      <c r="B341" s="1" t="s">
         <v>1386</v>
       </c>
       <c r="C341" t="s">
@@ -9224,7 +9224,7 @@
       <c r="A342" t="s">
         <v>550</v>
       </c>
-      <c r="B342" t="s">
+      <c r="B342" s="1" t="s">
         <v>551</v>
       </c>
       <c r="C342" t="s">
@@ -9235,7 +9235,7 @@
       <c r="A343" t="s">
         <v>550</v>
       </c>
-      <c r="B343" t="s">
+      <c r="B343" s="1" t="s">
         <v>553</v>
       </c>
       <c r="C343" t="s">
@@ -9246,7 +9246,7 @@
       <c r="A344" t="s">
         <v>550</v>
       </c>
-      <c r="B344" t="s">
+      <c r="B344" s="1" t="s">
         <v>692</v>
       </c>
       <c r="C344" t="s">
@@ -9257,7 +9257,7 @@
       <c r="A345" t="s">
         <v>550</v>
       </c>
-      <c r="B345" t="s">
+      <c r="B345" s="1" t="s">
         <v>1016</v>
       </c>
       <c r="C345" t="s">
@@ -9268,7 +9268,7 @@
       <c r="A346" t="s">
         <v>550</v>
       </c>
-      <c r="B346" t="s">
+      <c r="B346" s="1" t="s">
         <v>1047</v>
       </c>
       <c r="C346" t="s">
@@ -9279,7 +9279,7 @@
       <c r="A347" t="s">
         <v>550</v>
       </c>
-      <c r="B347" t="s">
+      <c r="B347" s="1" t="s">
         <v>1049</v>
       </c>
       <c r="C347" t="s">
@@ -9290,7 +9290,7 @@
       <c r="A348" t="s">
         <v>550</v>
       </c>
-      <c r="B348" t="s">
+      <c r="B348" s="1" t="s">
         <v>1074</v>
       </c>
       <c r="C348" t="s">

</xml_diff>

<commit_message>
feat: make the area card nicer to work with. Now the toggle is its own independent part, and if you click anywhere else on the areacard you expand the chevron undermenu. Also remove some console logs
</commit_message>
<xml_diff>
--- a/src/data/ruse-blocks.xlsx
+++ b/src/data/ruse-blocks.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2732" uniqueCount="1682">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2738" uniqueCount="1684">
   <si>
     <t>Дружба 1</t>
   </si>
@@ -5060,6 +5060,12 @@
   </si>
   <si>
     <t>ул. Бели хризантеми 9</t>
+  </si>
+  <si>
+    <t>ул. Солун 25</t>
+  </si>
+  <si>
+    <t>ул. Мехомия 7</t>
   </si>
 </sst>
 </file>
@@ -5451,10 +5457,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D991"/>
+  <dimension ref="A1:D993"/>
   <sheetFormatPr defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="15.5" customWidth="1"/>
+    <col min="1" max="1" width="17.8984375" customWidth="1"/>
     <col min="2" max="2" width="22.09765625" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="12.09765625" customWidth="1"/>
@@ -16308,7 +16314,7 @@
       <c r="A986" t="s">
         <v>151</v>
       </c>
-      <c r="B986" t="s">
+      <c r="B986" s="1" t="s">
         <v>260</v>
       </c>
       <c r="C986" t="s">
@@ -16330,7 +16336,7 @@
       <c r="A988" t="s">
         <v>151</v>
       </c>
-      <c r="B988" t="s">
+      <c r="B988" s="1" t="s">
         <v>923</v>
       </c>
       <c r="C988" t="s">
@@ -16341,7 +16347,7 @@
       <c r="A989" t="s">
         <v>151</v>
       </c>
-      <c r="B989" t="s">
+      <c r="B989" s="1" t="s">
         <v>1214</v>
       </c>
       <c r="C989" t="s">
@@ -16352,7 +16358,7 @@
       <c r="A990" t="s">
         <v>151</v>
       </c>
-      <c r="B990" t="s">
+      <c r="B990" s="1" t="s">
         <v>151</v>
       </c>
       <c r="C990" t="s">
@@ -16368,6 +16374,28 @@
       </c>
       <c r="C991" t="s">
         <v>1415</v>
+      </c>
+    </row>
+    <row r="992" spans="1:3">
+      <c r="A992" t="s">
+        <v>151</v>
+      </c>
+      <c r="B992" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="C992" t="s">
+        <v>1682</v>
+      </c>
+    </row>
+    <row r="993" spans="1:3">
+      <c r="A993" t="s">
+        <v>151</v>
+      </c>
+      <c r="B993" s="1" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C993" t="s">
+        <v>1683</v>
       </c>
     </row>
   </sheetData>

</xml_diff>